<commit_message>
Revert R2 Cache-Control change - breaks presigned URL signature
Cache-Control is a signed header in the R2 presigned upload URL.
Changing the value caused 403s on all R2 uploads. Reverted to
original value while a coordinated backend+frontend fix is planned.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documents/Eval Team.xlsx
+++ b/Documents/Eval Team.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\appli\source\repos\MemoryCharm\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA96E772-5417-412F-8B88-73A86145726C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9109B88E-FDFB-4940-BE37-A3BF1937EA53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-78" yWindow="0" windowWidth="11676" windowHeight="13758" xr2:uid="{6AC836F1-2141-447F-8EB3-3BE953C6A336}"/>
+    <workbookView xWindow="13560" yWindow="-18760" windowWidth="17280" windowHeight="9980" xr2:uid="{6AC836F1-2141-447F-8EB3-3BE953C6A336}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -56,9 +56,6 @@
     <t>19300 Splendor Ct</t>
   </si>
   <si>
-    <t>Jonestown, TX 78645</t>
-  </si>
-  <si>
     <t xml:space="preserve">KJ </t>
   </si>
   <si>
@@ -195,13 +192,16 @@
   </si>
   <si>
     <t>Seemakurthy</t>
+  </si>
+  <si>
+    <t>Jonestown, TX 78644</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,13 +217,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -239,9 +251,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -582,7 +596,9 @@
   <cols>
     <col min="2" max="2" width="12.62890625" customWidth="1"/>
     <col min="3" max="3" width="21.9453125" customWidth="1"/>
-    <col min="4" max="4" width="17.62890625" customWidth="1"/>
+    <col min="4" max="4" width="23.05078125" customWidth="1"/>
+    <col min="5" max="5" width="19.62890625" customWidth="1"/>
+    <col min="6" max="6" width="17.5234375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -601,10 +617,10 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>4</v>
@@ -612,163 +628,185 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
-        <v>6</v>
+      <c r="E2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2">
+        <v>3048180</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="D4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
         <v>24</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>26</v>
       </c>
-      <c r="E7" t="s">
-        <v>27</v>
+      <c r="F7">
+        <v>45126933</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
         <v>29</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>31</v>
       </c>
-      <c r="E8" t="s">
-        <v>32</v>
+      <c r="F8">
+        <v>48082363</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
         <v>36</v>
       </c>
-      <c r="B9" t="s">
-        <v>37</v>
-      </c>
       <c r="C9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
         <v>33</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>34</v>
       </c>
-      <c r="E9" t="s">
-        <v>35</v>
+      <c r="F9">
+        <v>127399</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
         <v>41</v>
       </c>
-      <c r="B10" t="s">
-        <v>42</v>
-      </c>
       <c r="C10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" t="s">
         <v>38</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>39</v>
       </c>
-      <c r="E10" t="s">
-        <v>40</v>
+      <c r="F10">
+        <v>4526461</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s">
         <v>46</v>
       </c>
-      <c r="B11" t="s">
-        <v>47</v>
-      </c>
       <c r="C11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" t="s">
         <v>43</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>44</v>
       </c>
-      <c r="E11" t="s">
-        <v>45</v>
+      <c r="F11">
+        <v>955856</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" t="s">
         <v>51</v>
       </c>
-      <c r="B12" t="s">
-        <v>52</v>
-      </c>
       <c r="C12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" t="s">
         <v>48</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>49</v>
       </c>
-      <c r="E12" t="s">
-        <v>50</v>
+      <c r="F12">
+        <v>78949127</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="mailto:joneskj7@hotmail.com" xr:uid="{D7DFA219-2C23-4704-A28E-05BF0536E1CE}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{C7B25296-6591-4B4C-AF27-1EFC1A7251DB}"/>

</xml_diff>